<commit_message>
Fix delivery note template vendor and A4 print
</commit_message>
<xml_diff>
--- a/maupgh.xlsx
+++ b/maupgh.xlsx
@@ -1,62 +1,70 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{115ADFEC-9A4F-46BF-89B8-43F63E53F75D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
-    <sheet name="E1" sheetId="15" r:id="rId1"/>
+    <sheet sheetId="15" name="E1" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase">'E1'!$A$15:$K$21</definedName>
+    <definedName name="_xlnm._FilterDatabase">E1!$A$15:$K$21</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'E1'!$A1:$H24</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
+    <t>BIÊN BẢN BÀN GIAO HÀNG HÓA</t>
+  </si>
+  <si>
+    <t>Ngày/ Date:</t>
+  </si>
+  <si>
+    <t>02/04/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   </t>
+  </si>
+  <si>
+    <t>Bên nhận:</t>
+  </si>
+  <si>
+    <t>Kho:</t>
+  </si>
+  <si>
+    <t>SS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Địa chỉ: </t>
+  </si>
+  <si>
+    <t>Lô CN 1-1, KCN Điềm Thụy, xã Điềm Thụy, tỉnh Thái Nguyên</t>
+  </si>
+  <si>
+    <t>Bên giao:</t>
+  </si>
+  <si>
     <t>CÔNG TY CỔ PHẦN PRECISION PACKAGING</t>
   </si>
   <si>
+    <t>MÃ NCC:</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
     <t>Cụm Công nghiệp Hạp Lĩnh, phường Khắc Niệm, tỉnh Bắc Ninh</t>
   </si>
   <si>
-    <t>BIÊN BẢN BÀN GIAO HÀNG HÓA</t>
-  </si>
-  <si>
-    <t>Ngày/ Date:</t>
-  </si>
-  <si>
-    <t>02/04/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   </t>
-  </si>
-  <si>
-    <t>Kho:</t>
-  </si>
-  <si>
-    <t>SS</t>
-  </si>
-  <si>
-    <t>Lô CN 1-1, KCN Điềm Thụy, xã Điềm Thụy, tỉnh Thái Nguyên</t>
-  </si>
-  <si>
-    <t>MÃ NCC:</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t>Hai bên thống nhất bàn giao số lượng hàng hóa như sau:</t>
   </si>
   <si>
@@ -90,143 +98,134 @@
     <t xml:space="preserve">V    </t>
   </si>
   <si>
+    <t>Giấy tờ kèm theo:</t>
+  </si>
+  <si>
     <t>BÊN GIAO</t>
   </si>
   <si>
     <t>BÊN NHẬN</t>
   </si>
   <si>
-    <t>Thủ kho
+    <t xml:space="preserve">Thủ kho
 (Ký, họ tên)</t>
   </si>
   <si>
-    <t>Người giao hàng
+    <t xml:space="preserve">Người giao hàng
 (Ký, họ tên)</t>
   </si>
   <si>
     <t>(Ký, họ tên)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Địa chỉ: </t>
-  </si>
-  <si>
-    <t>Bên giao:</t>
-  </si>
-  <si>
-    <t>Bên nhận:</t>
-  </si>
-  <si>
-    <t>Giấy tờ kèm theo:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="5">
     <numFmt numFmtId="164" formatCode="[$-1010000]d/m/yyyy;@"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0\ _₫_-;\-* #,##0\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="167" formatCode="#,##0.0000%;\-#,##0.0000%;"/>
-    <numFmt numFmtId="168" formatCode="#,##0.00;\(#,##0.00\)"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0 _₫_-;-* #,##0 _₫_-;_-* &quot;-&quot;?? _₫_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* (#,##0);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0000%;-#,##0.0000%;"/>
+    <numFmt numFmtId="168" formatCode="#,##0.00;(#,##0.00)"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <family val="1"/>
       <sz val="10"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
+    </font>
+    <font>
+      <family val="1"/>
       <sz val="12"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
       <b/>
+      <color indexed="8"/>
+      <family val="1"/>
       <sz val="18"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
       <color indexed="8"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
+      <family val="1"/>
       <sz val="11"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
       <color indexed="8"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
+      <family val="1"/>
       <sz val="12"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <b/>
       <color indexed="8"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <family val="1"/>
+      <sz val="13"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <color indexed="8"/>
+      <family val="1"/>
+      <sz val="13"/>
+      <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
-      <sz val="13"/>
       <color indexed="8"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <family val="1"/>
+      <sz val="16"/>
+      <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
+      <color indexed="8"/>
+      <family val="1"/>
+      <sz val="15"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <b/>
+      <color indexed="8"/>
+      <family val="1"/>
       <sz val="11"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <b/>
       <color indexed="8"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="13"/>
+      <family val="1"/>
+      <sz val="20"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <b/>
+      <family val="1"/>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <b/>
       <color indexed="8"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
+      <family val="1"/>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <i/>
       <color indexed="8"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color indexed="8"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="20"/>
-      <color indexed="8"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
+      <family val="1"/>
       <sz val="11"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -238,7 +237,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
+        <fgColor theme="4" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -329,7 +328,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -344,26 +343,29 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -373,31 +375,37 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -418,10 +426,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -430,40 +435,34 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -471,15 +470,6 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -783,13 +773,13 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U22"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A2:U22"/>
+  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="9.125" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="9.875" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.625" style="2" customWidth="1"/>
@@ -804,234 +794,232 @@
     <col min="11" max="11" width="30.125" style="1" customWidth="1"/>
     <col min="12" max="12" width="24.875" style="1" customWidth="1"/>
     <col min="13" max="13" width="16.375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="9.125" style="1" customWidth="1"/>
-    <col min="15" max="16384" width="9.125" style="1"/>
+    <col min="14" max="16384" width="9.125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:21" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-    </row>
-    <row r="3" spans="1:21" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="48"/>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
-    </row>
-    <row r="4" spans="1:21" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="7"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="7"/>
-    </row>
-    <row r="5" spans="1:21" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="5"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="14"/>
-    </row>
-    <row r="6" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="41" t="s">
+    <row r="2" ht="24.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+    </row>
+    <row r="3" ht="21.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+    </row>
+    <row r="4" ht="16.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="6"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="6"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="11"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="15"/>
+    </row>
+    <row r="6" ht="22.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+    </row>
+    <row r="8" ht="20.25" customHeight="1" spans="7:21" x14ac:dyDescent="0.25">
+      <c r="G8" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="H8" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="41"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="41"/>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="41"/>
-    </row>
-    <row r="8" spans="1:21" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G8" s="50" t="s">
+      <c r="U8" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H8" s="49" t="s">
+    </row>
+    <row r="9" ht="21.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="U8" s="1" t="s">
+      <c r="B9" s="17"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="1:21" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17" t="s">
+      <c r="H9" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="H9" s="17" t="s">
+    </row>
+    <row r="10" ht="36.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="21" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="1:21" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-    </row>
-    <row r="11" spans="1:21" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="21" t="s">
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+    </row>
+    <row r="11" ht="21.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A11" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="H11" s="22" t="s">
+      <c r="B11" s="17" t="s">
         <v>10</v>
       </c>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H11" s="25" t="s">
+        <v>12</v>
+      </c>
       <c r="S11" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="19" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" ht="34.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="29"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+    </row>
+    <row r="15" ht="39" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" s="31" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="H15" s="31" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" ht="46.5" customHeight="1" spans="1:10" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="34">
         <v>1</v>
       </c>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24"/>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A13" s="25" t="s">
+      <c r="B16" s="35"/>
+      <c r="C16" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="26"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="27"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-    </row>
-    <row r="15" spans="1:21" s="3" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="28" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="C15" s="29" t="s">
-        <v>15</v>
-      </c>
-      <c r="D15" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="E15" s="28" t="s">
-        <v>17</v>
-      </c>
-      <c r="F15" s="28" t="s">
-        <v>18</v>
-      </c>
-      <c r="G15" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="H15" s="30" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" s="31" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="32">
-        <v>1</v>
-      </c>
-      <c r="B16" s="33"/>
-      <c r="C16" s="34" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="E16" s="35"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="36"/>
-      <c r="H16" s="28"/>
-      <c r="I16" s="37"/>
-      <c r="J16" s="37"/>
-    </row>
-    <row r="17" spans="1:17" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="42" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="43"/>
-      <c r="C17" s="43"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="44"/>
-      <c r="G17" s="38"/>
-      <c r="H17" s="39"/>
+      <c r="D16" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="37"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="39"/>
+      <c r="J16" s="39"/>
+    </row>
+    <row r="17" ht="38.25" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="40"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="41"/>
+      <c r="G17" s="42"/>
+      <c r="H17" s="43"/>
       <c r="M17" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" s="26"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="40"/>
-      <c r="G18" s="40"/>
-      <c r="H18" s="40"/>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" ht="26.25" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="29"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="44"/>
+      <c r="G18" s="44"/>
+      <c r="H18" s="44"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="45" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B19" s="45"/>
       <c r="C19" s="45"/>
       <c r="D19" s="45"/>
       <c r="E19" s="45"/>
       <c r="F19" s="45" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G19" s="45"/>
       <c r="H19" s="45"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="45"/>
       <c r="B20" s="45"/>
       <c r="C20" s="45"/>
@@ -1041,44 +1029,44 @@
       <c r="G20" s="45"/>
       <c r="H20" s="45"/>
     </row>
-    <row r="21" spans="1:17" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" ht="60" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="46" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B21" s="47"/>
       <c r="C21" s="47"/>
       <c r="D21" s="46" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E21" s="46"/>
       <c r="F21" s="47" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G21" s="47"/>
       <c r="H21" s="47"/>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="22" spans="17:17" x14ac:dyDescent="0.25">
       <c r="Q22" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A15:K21" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A15:K21"/>
   <mergeCells count="11">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="F19:H19"/>
     <mergeCell ref="A20:E20"/>
     <mergeCell ref="F20:H20"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="D21:E21"/>
     <mergeCell ref="F21:H21"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="F19:H19"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.26" right="0.196850393700787" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
-  <pageSetup paperSize="9" scale="59" fitToHeight="0" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
+  <pageMargins left="0.26" right="0.196850393700787" top="0.748031496062992" bottom="0.748031496062992" header="0.31496062992126" footer="0.31496062992126"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="59" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>